<commit_message>
fix(e2e): harness HARN lane IDs, SQL cleanup, genexpert template bind-mount
- Add analyzer-harness-lane-data.sql + load on --analyzers=full
- Reset HARN-* DB residue in file-import-e2e.sql (psql ON_ERROR_STOP in workflows)
- Mount e2e-fixtures/genexpert_astm.json for ASTM simulator (no submodule bump)
- QuantStudio fixture + Playwright expectations for HARN-QS7 accessions
- Docs: LANE-IDENTIFIERS.md, roadmap/mock remediation alignment

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/frontend/playwright/fixtures/quantstudio-e2e-results.xlsx
+++ b/frontend/playwright/fixtures/quantstudio-e2e-results.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>E2E001</t>
+          <t>HARN-QS7-2026-00001</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,7 +531,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>E2E002</t>
+          <t>HARN-QS7-2026-00002</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>E2E003</t>
+          <t>HARN-QS7-2026-00003</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>E2E004</t>
+          <t>HARN-QS7-2026-00004</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>E2E005</t>
+          <t>HARN-QS7-2026-00005</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>E2E007</t>
+          <t>HARN-QS7-2026-00007</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">

</xml_diff>